<commit_message>
fix: enable CI running
</commit_message>
<xml_diff>
--- a/TDD_examples/CASE_1_ITER_like_LTS/conductor_1_input.xlsx
+++ b/TDD_examples/CASE_1_ITER_like_LTS/conductor_1_input.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="CHAN" sheetId="1" state="visible" r:id="rId2"/>
@@ -557,12 +557,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -570,7 +570,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -582,7 +582,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -602,10 +602,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
@@ -615,10 +611,6 @@
       <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -686,7 +678,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -704,7 +696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6"/>
       <c r="B2" s="5"/>
       <c r="D2" s="7" t="s">
@@ -719,7 +711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
         <f aca="false">[1]TRANSIENT!A$2</f>
         <v>Variable name</v>
@@ -745,7 +737,7 @@
         <v>CHAN_2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -765,7 +757,7 @@
         <v>0.00036965</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -785,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -805,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -825,7 +817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -845,7 +837,7 @@
         <v>0.00032676</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -865,7 +857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
@@ -885,7 +877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
@@ -905,7 +897,7 @@
         <v>0.313</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>25</v>
       </c>
@@ -925,7 +917,7 @@
         <v>-99</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
         <v>28</v>
       </c>
@@ -945,7 +937,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
@@ -955,16 +947,16 @@
       <c r="C14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="11" t="b">
+      <c r="E14" s="2" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F14" s="11" t="b">
+      <c r="F14" s="2" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -998,7 +990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1018,7 +1010,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
@@ -1038,7 +1030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1051,11 +1043,11 @@
       <c r="D19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="11" t="b">
+      <c r="E19" s="2" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F19" s="11" t="b">
+      <c r="F19" s="2" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1088,7 +1080,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>42</v>
       </c>
@@ -1104,7 +1096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -1116,7 +1108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
         <f aca="false">CHAN!A3</f>
         <v>Variable name</v>
@@ -1138,7 +1130,7 @@
         <v>STACK_0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>3</v>
       </c>
@@ -1151,11 +1143,11 @@
       <c r="D4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -1189,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
         <v>21</v>
       </c>
@@ -1206,7 +1198,7 @@
         <v>0.9699</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>45</v>
       </c>
@@ -1223,7 +1215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
         <v>48</v>
       </c>
@@ -1238,7 +1230,7 @@
       </c>
       <c r="E9" s="9"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>50</v>
       </c>
@@ -1253,7 +1245,7 @@
       </c>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
         <v>52</v>
       </c>
@@ -1268,7 +1260,7 @@
       </c>
       <c r="E11" s="9"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
         <v>54</v>
       </c>
@@ -1283,7 +1275,7 @@
       </c>
       <c r="E12" s="9"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
         <v>56</v>
       </c>
@@ -1298,7 +1290,7 @@
       </c>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>58</v>
       </c>
@@ -1313,7 +1305,7 @@
       </c>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
         <v>60</v>
       </c>
@@ -1328,7 +1320,7 @@
       </c>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
         <v>62</v>
       </c>
@@ -1343,7 +1335,7 @@
       </c>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
         <v>64</v>
       </c>
@@ -1358,7 +1350,7 @@
       </c>
       <c r="E17" s="9"/>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
         <v>66</v>
       </c>
@@ -1368,12 +1360,12 @@
       <c r="C18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>67</v>
       </c>
       <c r="E18" s="9"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
         <v>68</v>
       </c>
@@ -1388,7 +1380,7 @@
       </c>
       <c r="E19" s="9"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
         <v>70</v>
       </c>
@@ -1403,7 +1395,7 @@
       </c>
       <c r="E20" s="9"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
         <v>72</v>
       </c>
@@ -1420,7 +1412,7 @@
         <v>170360000000000</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
         <v>75</v>
       </c>
@@ -1437,7 +1429,7 @@
         <v>30.23</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>77</v>
       </c>
@@ -1454,7 +1446,7 @@
         <v>16.73</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
         <v>79</v>
       </c>
@@ -1471,7 +1463,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
         <v>81</v>
       </c>
@@ -1489,7 +1481,7 @@
         <v>1E-005</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
         <v>40</v>
       </c>
@@ -1502,7 +1494,7 @@
       <c r="D26" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="11" t="b">
+      <c r="E26" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1534,7 +1526,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>85</v>
       </c>
@@ -1550,7 +1542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -1562,7 +1554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
         <f aca="false">CHAN!A3</f>
         <v>Variable name</v>
@@ -1584,7 +1576,7 @@
         <v>STR_MIX_1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1602,7 +1594,7 @@
         <v>0.000753951765</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1619,7 +1611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1636,7 +1628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1653,7 +1645,7 @@
         <v>0.9699</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>91</v>
       </c>
@@ -1670,7 +1662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>93</v>
       </c>
@@ -1687,7 +1679,7 @@
         <v>2.0846</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -1700,11 +1692,11 @@
       <c r="D10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="13" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>97</v>
       </c>
@@ -1721,7 +1713,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>99</v>
       </c>
@@ -1739,7 +1731,7 @@
         <v>0.000822</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>101</v>
       </c>
@@ -1756,7 +1748,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>103</v>
       </c>
@@ -1774,7 +1766,7 @@
         <v>0.000821</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>105</v>
       </c>
@@ -1791,7 +1783,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>108</v>
       </c>
@@ -1804,11 +1796,11 @@
       <c r="D16" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="13" t="n">
         <v>197.71</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>110</v>
       </c>
@@ -1825,7 +1817,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>113</v>
       </c>
@@ -1842,7 +1834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>72</v>
       </c>
@@ -1859,7 +1851,7 @@
         <v>121508000000</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>75</v>
       </c>
@@ -1876,7 +1868,7 @@
         <v>32.35</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>77</v>
       </c>
@@ -1893,7 +1885,7 @@
         <v>16.22</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
         <v>79</v>
       </c>
@@ -1910,7 +1902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>81</v>
       </c>
@@ -1928,7 +1920,7 @@
         <v>1E-005</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -1941,8 +1933,9 @@
       <c r="D24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E24" s="15" t="n">
-        <v>1</v>
+      <c r="E24" s="2" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1973,7 +1966,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>115</v>
       </c>
@@ -1989,11 +1982,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>117</v>
       </c>
       <c r="E2" s="4" t="n">
@@ -2001,7 +1994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
         <f aca="false">CHAN!A3</f>
         <v>Variable name</v>
@@ -2023,7 +2016,7 @@
         <v>STR_STAB_0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2036,11 +2029,11 @@
       <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -2057,7 +2050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -2074,7 +2067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -2091,7 +2084,7 @@
         <v>0.9699</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>105</v>
       </c>
@@ -2104,11 +2097,11 @@
       <c r="D8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="13" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>108</v>
       </c>
@@ -2121,11 +2114,11 @@
       <c r="D9" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="14" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>40</v>
       </c>
@@ -2138,7 +2131,7 @@
       <c r="D10" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="11" t="b">
+      <c r="E10" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2171,7 +2164,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>118</v>
       </c>
@@ -2187,7 +2180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -2199,7 +2192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
         <f aca="false">CHAN!A3</f>
         <v>Variable name</v>
@@ -2221,7 +2214,7 @@
         <v>Z_JACKET_1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>121</v>
       </c>
@@ -2239,7 +2232,7 @@
         <v>0.00030699</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
@@ -2256,7 +2249,7 @@
         <v>0.00027966</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -2273,7 +2266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -2290,7 +2283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>126</v>
       </c>
@@ -2307,7 +2300,7 @@
         <v>0.1288</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>128</v>
       </c>
@@ -2324,7 +2317,7 @@
         <v>0.1357</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -2337,11 +2330,11 @@
       <c r="D10" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="14" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
         <v>131</v>
       </c>
@@ -2354,11 +2347,11 @@
       <c r="D11" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="14" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>134</v>
       </c>
@@ -2371,11 +2364,11 @@
       <c r="D12" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="14" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -2392,7 +2385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>137</v>
       </c>
@@ -2405,11 +2398,11 @@
       <c r="D14" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="15" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>140</v>
       </c>
@@ -2426,7 +2419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>40</v>
       </c>

</xml_diff>